<commit_message>
fix percent issue in Excel
</commit_message>
<xml_diff>
--- a/Librairies/TEP-AltiumLib-Passives-RLC.xlsx
+++ b/Librairies/TEP-AltiumLib-Passives-RLC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lecegeplimoilou-my.sharepoint.com/personal/kevin_cotton_cegeplimoilou_ca/Documents/_Cours-TGE/Altium/243-TEP_Altium-Lib/Librairies/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1595" documentId="13_ncr:1_{550D3E46-E4B6-4165-A45B-7D583CCE157E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EBF0353B-B995-417F-8815-1524ADBCECDB}"/>
+  <xr:revisionPtr revIDLastSave="1600" documentId="13_ncr:1_{550D3E46-E4B6-4165-A45B-7D583CCE157E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67D1AD32-6B5E-4CA3-88EF-6BBB2E4DD030}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="16490" windowHeight="10260" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1460" yWindow="430" windowWidth="16490" windowHeight="10260" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cap" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1330" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1335" uniqueCount="503">
   <si>
     <t>Comment</t>
   </si>
@@ -1546,6 +1546,12 @@
   </si>
   <si>
     <t>L_4040[1515]</t>
+  </si>
+  <si>
+    <t>30%</t>
+  </si>
+  <si>
+    <t>25%</t>
   </si>
 </sst>
 </file>
@@ -5935,8 +5941,8 @@
       <c r="I2" t="s">
         <v>462</v>
       </c>
-      <c r="J2" s="7">
-        <v>0.25</v>
+      <c r="J2" s="7" t="s">
+        <v>502</v>
       </c>
       <c r="K2" t="s">
         <v>495</v>
@@ -5982,8 +5988,8 @@
       <c r="I3" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="J3" s="7">
-        <v>0.25</v>
+      <c r="J3" s="7" t="s">
+        <v>502</v>
       </c>
       <c r="K3" t="s">
         <v>140</v>
@@ -6029,8 +6035,8 @@
       <c r="I4" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="J4" s="7">
-        <v>0.25</v>
+      <c r="J4" s="7" t="s">
+        <v>502</v>
       </c>
       <c r="K4" t="s">
         <v>144</v>
@@ -6076,8 +6082,8 @@
       <c r="I5" t="s">
         <v>456</v>
       </c>
-      <c r="J5" s="9">
-        <v>0.1</v>
+      <c r="J5" s="7" t="s">
+        <v>133</v>
       </c>
       <c r="K5" t="s">
         <v>205</v>
@@ -6167,8 +6173,8 @@
       <c r="I7" t="s">
         <v>462</v>
       </c>
-      <c r="J7" s="9">
-        <v>0.3</v>
+      <c r="J7" s="7" t="s">
+        <v>501</v>
       </c>
       <c r="K7" t="s">
         <v>493</v>

</xml_diff>